<commit_message>
update NCR weekly dashboard data
</commit_message>
<xml_diff>
--- a/docs/reports/NCR_Kavach_Unified_KPI_Jun22-Jun28.xlsx
+++ b/docs/reports/NCR_Kavach_Unified_KPI_Jun22-Jun28.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Unified KPI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Daily Breakdown" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="EB Detail" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Mode Degradation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KM Verification" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Methodology" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10063,7 +10063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L214"/>
+  <dimension ref="A1:M214"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10141,6 +10141,11 @@
           <t>Valid Trip?</t>
         </is>
       </c>
+      <c r="M5" s="14" t="inlineStr">
+        <is>
+          <t>Loco Travel</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -10197,6 +10202,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M6" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -10253,6 +10263,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M7" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -10309,6 +10324,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M8" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -10365,6 +10385,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M9" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -10421,6 +10446,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M10" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -10477,6 +10507,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M11" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -10533,6 +10568,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M12" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -10589,6 +10629,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M13" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -10645,6 +10690,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M14" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -10701,6 +10751,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -10757,6 +10812,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -10813,6 +10873,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -10869,6 +10934,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M18" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -10925,6 +10995,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M19" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -10981,6 +11056,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M20" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -11037,6 +11117,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M21" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -11093,6 +11178,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M22" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -11149,6 +11239,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M23" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -11205,6 +11300,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M24" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -11261,6 +11361,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M25" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -11317,6 +11422,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M26" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -11373,6 +11483,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M27" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -11429,6 +11544,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M28" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -11485,6 +11605,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M29" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -11541,6 +11666,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M30" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -11597,6 +11727,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M31" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -11653,6 +11788,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M32" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -11709,6 +11849,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M33" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -11765,6 +11910,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M34" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -11821,6 +11971,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M35" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -11877,6 +12032,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M36" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -11933,6 +12093,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M37" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -11989,6 +12154,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M38" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="34" t="inlineStr">
@@ -12045,6 +12215,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M39" s="16" t="inlineStr">
+        <is>
+          <t>LC545, Chhata, LC540, Ajhai</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="34" t="inlineStr">
@@ -12101,6 +12276,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M40" s="16" t="inlineStr">
+        <is>
+          <t>LC545, Chhata, LC540, Ajhai</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
@@ -12157,6 +12337,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M41" s="16" t="inlineStr">
+        <is>
+          <t>LC545, Chhata, LC540, Ajhai</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="34" t="inlineStr">
@@ -12213,6 +12398,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M42" s="16" t="inlineStr">
+        <is>
+          <t>LC545, Chhata, LC540, Ajhai</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="16" t="inlineStr">
@@ -12269,6 +12459,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M43" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="16" t="inlineStr">
@@ -12325,6 +12520,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M44" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="16" t="inlineStr">
@@ -12381,6 +12581,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M45" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr">
@@ -12437,6 +12642,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr">
@@ -12493,6 +12703,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr">
@@ -12549,6 +12764,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr">
@@ -12605,6 +12825,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr">
@@ -12661,6 +12886,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr">
@@ -12717,6 +12947,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr">
@@ -12773,6 +13008,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
@@ -12829,6 +13069,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
@@ -12885,6 +13130,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr">
@@ -12941,6 +13191,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr">
@@ -12997,6 +13248,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M56" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr">
@@ -13053,6 +13309,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M57" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr">
@@ -13109,6 +13370,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M58" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr">
@@ -13165,6 +13431,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M59" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr">
@@ -13221,6 +13492,7 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr">
@@ -13277,6 +13549,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M61" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="16" t="inlineStr">
@@ -13333,6 +13610,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M62" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="16" t="inlineStr">
@@ -13389,6 +13671,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M63" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="16" t="inlineStr">
@@ -13445,6 +13732,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M64" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
@@ -13501,6 +13793,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M65" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr">
@@ -13557,6 +13854,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M66" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr">
@@ -13613,6 +13915,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M67" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
@@ -13669,6 +13976,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M68" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr">
@@ -13725,6 +14037,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M69" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr">
@@ -13781,6 +14098,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M70" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="16" t="inlineStr">
@@ -13837,6 +14159,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M71" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
@@ -13893,6 +14220,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M72" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="16" t="inlineStr">
@@ -13949,6 +14281,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M73" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr">
@@ -14005,6 +14342,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M74" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr">
@@ -14061,6 +14403,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M75" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr">
@@ -14117,6 +14464,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M76" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
@@ -14173,6 +14525,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M77" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr">
@@ -14229,6 +14586,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M78" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr">
@@ -14285,6 +14647,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M79" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="16" t="inlineStr">
@@ -14341,6 +14708,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M80" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="16" t="inlineStr">
@@ -14397,6 +14769,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M81" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="16" t="inlineStr">
@@ -14453,6 +14830,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M82" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -14509,6 +14891,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M83" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="16" t="inlineStr">
@@ -14565,6 +14952,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M84" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="16" t="inlineStr">
@@ -14621,6 +15013,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M85" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="16" t="inlineStr">
@@ -14677,6 +15074,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M86" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="16" t="inlineStr">
@@ -14733,6 +15135,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M87" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="16" t="inlineStr">
@@ -14789,6 +15196,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M88" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="16" t="inlineStr">
@@ -14845,6 +15257,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M89" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="16" t="inlineStr">
@@ -14901,6 +15318,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M90" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="16" t="inlineStr">
@@ -14957,6 +15379,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M91" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="16" t="inlineStr">
@@ -15013,6 +15440,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M92" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="16" t="inlineStr">
@@ -15069,6 +15501,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M93" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="16" t="inlineStr">
@@ -15125,6 +15562,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M94" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="16" t="inlineStr">
@@ -15181,6 +15623,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M95" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="16" t="inlineStr">
@@ -15237,6 +15684,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M96" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="16" t="inlineStr">
@@ -15293,6 +15745,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M97" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="16" t="inlineStr">
@@ -15349,6 +15806,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M98" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="16" t="inlineStr">
@@ -15405,6 +15867,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M99" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="16" t="inlineStr">
@@ -15461,6 +15928,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M100" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="16" t="inlineStr">
@@ -15517,6 +15989,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M101" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="16" t="inlineStr">
@@ -15573,6 +16050,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M102" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="16" t="inlineStr">
@@ -15629,6 +16111,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M103" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="16" t="inlineStr">
@@ -15685,6 +16172,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M104" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="16" t="inlineStr">
@@ -15741,6 +16233,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M105" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="16" t="inlineStr">
@@ -15797,6 +16294,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M106" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="34" t="inlineStr">
@@ -15853,6 +16355,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M107" s="16" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="34" t="inlineStr">
@@ -15909,6 +16412,7 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M108" s="16" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="16" t="inlineStr">
@@ -15965,6 +16469,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M109" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="16" t="inlineStr">
@@ -16021,6 +16530,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M110" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="16" t="inlineStr">
@@ -16077,6 +16591,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M111" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="16" t="inlineStr">
@@ -16133,6 +16652,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M112" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="16" t="inlineStr">
@@ -16189,6 +16713,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M113" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="16" t="inlineStr">
@@ -16245,6 +16774,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M114" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="16" t="inlineStr">
@@ -16301,6 +16835,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M115" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="16" t="inlineStr">
@@ -16357,6 +16896,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M116" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="16" t="inlineStr">
@@ -16413,6 +16957,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M117" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="16" t="inlineStr">
@@ -16469,6 +17018,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M118" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="16" t="inlineStr">
@@ -16525,6 +17079,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M119" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="16" t="inlineStr">
@@ -16581,6 +17140,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M120" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="16" t="inlineStr">
@@ -16637,6 +17201,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M121" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="16" t="inlineStr">
@@ -16693,6 +17262,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M122" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="16" t="inlineStr">
@@ -16749,6 +17323,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M123" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="16" t="inlineStr">
@@ -16805,6 +17384,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M124" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="16" t="inlineStr">
@@ -16861,6 +17445,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M125" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="16" t="inlineStr">
@@ -16917,6 +17506,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M126" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="16" t="inlineStr">
@@ -16973,6 +17567,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M127" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="16" t="inlineStr">
@@ -17029,6 +17628,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M128" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="16" t="inlineStr">
@@ -17085,6 +17689,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M129" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="16" t="inlineStr">
@@ -17141,6 +17750,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M130" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="16" t="inlineStr">
@@ -17197,6 +17811,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M131" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="16" t="inlineStr">
@@ -17253,6 +17872,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M132" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="16" t="inlineStr">
@@ -17309,6 +17933,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M133" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="16" t="inlineStr">
@@ -17365,6 +17994,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M134" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="16" t="inlineStr">
@@ -17421,6 +18055,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M135" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="16" t="inlineStr">
@@ -17477,6 +18116,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M136" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="16" t="inlineStr">
@@ -17533,6 +18177,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M137" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="16" t="inlineStr">
@@ -17589,6 +18238,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M138" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="16" t="inlineStr">
@@ -17645,6 +18299,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M139" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="16" t="inlineStr">
@@ -17701,6 +18360,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M140" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="16" t="inlineStr">
@@ -17757,6 +18421,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M141" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="16" t="inlineStr">
@@ -17813,6 +18482,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M142" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="16" t="inlineStr">
@@ -17869,6 +18543,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M143" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="16" t="inlineStr">
@@ -17925,6 +18604,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M144" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="16" t="inlineStr">
@@ -17981,6 +18665,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M145" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="16" t="inlineStr">
@@ -18037,6 +18726,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M146" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="16" t="inlineStr">
@@ -18093,6 +18787,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M147" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="16" t="inlineStr">
@@ -18149,6 +18848,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M148" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="16" t="inlineStr">
@@ -18205,6 +18909,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M149" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="16" t="inlineStr">
@@ -18261,6 +18970,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M150" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="16" t="inlineStr">
@@ -18317,6 +19031,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M151" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="16" t="inlineStr">
@@ -18373,6 +19092,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M152" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="16" t="inlineStr">
@@ -18429,6 +19153,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M153" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="16" t="inlineStr">
@@ -18485,6 +19214,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M154" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="16" t="inlineStr">
@@ -18541,6 +19275,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M155" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="16" t="inlineStr">
@@ -18597,6 +19336,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M156" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="16" t="inlineStr">
@@ -18653,6 +19397,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M157" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="16" t="inlineStr">
@@ -18709,6 +19458,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M158" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="16" t="inlineStr">
@@ -18765,6 +19519,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M159" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="16" t="inlineStr">
@@ -18821,6 +19580,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M160" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="16" t="inlineStr">
@@ -18877,6 +19641,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M161" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="16" t="inlineStr">
@@ -18933,6 +19702,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M162" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="16" t="inlineStr">
@@ -18989,6 +19763,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M163" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="16" t="inlineStr">
@@ -19045,6 +19824,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M164" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="16" t="inlineStr">
@@ -19101,6 +19885,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M165" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="16" t="inlineStr">
@@ -19157,6 +19946,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M166" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="16" t="inlineStr">
@@ -19213,6 +20007,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M167" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="16" t="inlineStr">
@@ -19269,6 +20068,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M168" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="16" t="inlineStr">
@@ -19325,6 +20129,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M169" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="16" t="inlineStr">
@@ -19381,6 +20190,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M170" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="16" t="inlineStr">
@@ -19437,6 +20251,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M171" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="16" t="inlineStr">
@@ -19493,6 +20312,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M172" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="16" t="inlineStr">
@@ -19549,6 +20373,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M173" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="16" t="inlineStr">
@@ -19605,6 +20434,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M174" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="16" t="inlineStr">
@@ -19661,6 +20495,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M175" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="16" t="inlineStr">
@@ -19717,6 +20556,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M176" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="16" t="inlineStr">
@@ -19773,6 +20617,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M177" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="16" t="inlineStr">
@@ -19829,6 +20678,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M178" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="16" t="inlineStr">
@@ -19885,6 +20739,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M179" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="16" t="inlineStr">
@@ -19941,6 +20800,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M180" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="16" t="inlineStr">
@@ -19997,6 +20861,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M181" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="16" t="inlineStr">
@@ -20053,6 +20922,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M182" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="16" t="inlineStr">
@@ -20109,6 +20983,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M183" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="16" t="inlineStr">
@@ -20165,6 +21044,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M184" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="16" t="inlineStr">
@@ -20221,6 +21105,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M185" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="16" t="inlineStr">
@@ -20277,6 +21166,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M186" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="16" t="inlineStr">
@@ -20333,6 +21227,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M187" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="16" t="inlineStr">
@@ -20389,6 +21288,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M188" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="16" t="inlineStr">
@@ -20445,6 +21349,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M189" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="16" t="inlineStr">
@@ -20501,6 +21410,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M190" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="16" t="inlineStr">
@@ -20557,6 +21471,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M191" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="16" t="inlineStr">
@@ -20613,6 +21532,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M192" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="16" t="inlineStr">
@@ -20669,6 +21593,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M193" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="16" t="inlineStr">
@@ -20725,6 +21654,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M194" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="16" t="inlineStr">
@@ -20781,6 +21715,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M195" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="16" t="inlineStr">
@@ -20837,6 +21776,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M196" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="16" t="inlineStr">
@@ -20893,6 +21837,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M197" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="16" t="inlineStr">
@@ -20949,6 +21898,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M198" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="16" t="inlineStr">
@@ -21005,6 +21959,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M199" s="16" t="inlineStr">
+        <is>
+          <t>LC545, Chhata</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="16" t="inlineStr">
@@ -21061,6 +22020,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M200" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="16" t="inlineStr">
@@ -21117,6 +22081,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M201" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="16" t="inlineStr">
@@ -21173,6 +22142,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M202" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="16" t="inlineStr">
@@ -21229,6 +22203,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M203" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="16" t="inlineStr">
@@ -21285,6 +22264,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M204" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="16" t="inlineStr">
@@ -21341,6 +22325,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M205" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="16" t="inlineStr">
@@ -21397,6 +22386,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M206" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="16" t="inlineStr">
@@ -21453,6 +22447,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M207" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="16" t="inlineStr">
@@ -21509,6 +22508,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M208" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="16" t="inlineStr">
@@ -21565,6 +22569,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M209" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="16" t="inlineStr">
@@ -21621,6 +22630,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M210" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="16" t="inlineStr">
@@ -21677,6 +22691,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M211" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="16" t="inlineStr">
@@ -21733,6 +22752,11 @@
           <t>Valid</t>
         </is>
       </c>
+      <c r="M212" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="34" t="inlineStr">
@@ -21789,6 +22813,11 @@
           <t>Non-Valid</t>
         </is>
       </c>
+      <c r="M213" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="16" t="inlineStr">
@@ -21843,6 +22872,11 @@
       <c r="L214" s="16" t="inlineStr">
         <is>
           <t>Valid</t>
+        </is>
+      </c>
+      <c r="M214" s="16" t="inlineStr">
+        <is>
+          <t>LC563, LC562, LC561, LC559, LC557, LC556, LC555, LC553, LC551, LC545, Chhata, LC540, Ajhai, LC535, Vrindavan Road, BCH</t>
         </is>
       </c>
     </row>

</xml_diff>